<commit_message>
Add real timeout protection to Compounder_Scanner.py - fixes the stuck-fetch issue, plus restore the rate-limiting/progress code
</commit_message>
<xml_diff>
--- a/COMPOUNDER_WATCHLIST.xlsx
+++ b/COMPOUNDER_WATCHLIST.xlsx
@@ -471,21 +471,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AQYLON</t>
+          <t>MAHLIFE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>50</v>
+        <v>37.22</v>
       </c>
       <c r="C2" t="n">
-        <v>-74.47</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
+        <v>-21.55</v>
+      </c>
+      <c r="D2" t="n">
+        <v>12.04</v>
+      </c>
       <c r="E2" t="n">
-        <v>24294.8</v>
+        <v>2909.5</v>
       </c>
       <c r="F2" t="n">
-        <v>84.51000000000001</v>
+        <v>33.13</v>
       </c>
       <c r="G2" t="n">
         <v>100</v>
@@ -509,7 +511,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35.42</v>
+        <v>35.45</v>
       </c>
       <c r="C3" t="n">
         <v>-6.34</v>
@@ -545,7 +547,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28.81</v>
+        <v>30.34</v>
       </c>
       <c r="C4" t="n">
         <v>279.21</v>
@@ -575,30 +577,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CASTROLIND</t>
+          <t>SIL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21.09</v>
+        <v>22.84</v>
       </c>
       <c r="C5" t="n">
-        <v>-12.35</v>
-      </c>
-      <c r="D5" t="n">
-        <v>57</v>
-      </c>
+        <v>-25.51</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>25</v>
+        <v>1734.9</v>
       </c>
       <c r="F5" t="n">
-        <v>28.37</v>
+        <v>40.62</v>
       </c>
       <c r="G5" t="n">
         <v>100</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -611,30 +611,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>OFSS</t>
+          <t>CASTROLIND</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20.56</v>
+        <v>21.49</v>
       </c>
       <c r="C6" t="n">
-        <v>7.68</v>
+        <v>-12.35</v>
       </c>
       <c r="D6" t="n">
-        <v>49.9</v>
+        <v>57</v>
       </c>
       <c r="E6" t="n">
-        <v>68.7</v>
+        <v>25</v>
       </c>
       <c r="F6" t="n">
-        <v>34.34</v>
+        <v>28.37</v>
       </c>
       <c r="G6" t="n">
         <v>100</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Oil &amp; Gas</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -647,28 +647,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ATHERENERG</t>
+          <t>OFSS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19.97</v>
+        <v>21.2</v>
       </c>
       <c r="C7" t="n">
-        <v>265.44</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>7.68</v>
+      </c>
+      <c r="D7" t="n">
+        <v>49.9</v>
+      </c>
       <c r="E7" t="n">
-        <v>88.8</v>
+        <v>68.7</v>
       </c>
       <c r="F7" t="n">
-        <v>48.2</v>
+        <v>34.34</v>
       </c>
       <c r="G7" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -681,24 +683,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CPPLUS</t>
+          <t>ATHERENERG</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18.16</v>
+        <v>20.73</v>
       </c>
       <c r="C8" t="n">
-        <v>217.16</v>
+        <v>265.44</v>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>89.5</v>
+        <v>88.8</v>
       </c>
       <c r="F8" t="n">
-        <v>44.86</v>
+        <v>48.2</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -715,21 +717,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SETL</t>
+          <t>CPPLUS</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17.23</v>
+        <v>18.97</v>
       </c>
       <c r="C9" t="n">
-        <v>65.77</v>
+        <v>217.16</v>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>43.1</v>
+        <v>89.5</v>
       </c>
       <c r="F9" t="n">
-        <v>52.75</v>
+        <v>44.86</v>
       </c>
       <c r="G9" t="n">
         <v>100</v>
@@ -749,21 +751,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>INDSWFTLAB</t>
+          <t>SETL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16.98</v>
+        <v>17.17</v>
       </c>
       <c r="C10" t="n">
-        <v>56.94</v>
+        <v>65.77</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>25.4</v>
+        <v>43.1</v>
       </c>
       <c r="F10" t="n">
-        <v>56.57</v>
+        <v>52.75</v>
       </c>
       <c r="G10" t="n">
         <v>100</v>
@@ -787,7 +789,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16.27</v>
+        <v>16.76</v>
       </c>
       <c r="C11" t="n">
         <v>-23.66</v>
@@ -819,24 +821,24 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PVP</t>
+          <t>INDSWFTLAB</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>14.8</v>
+        <v>16.55</v>
       </c>
       <c r="C12" t="n">
-        <v>56.74</v>
+        <v>56.94</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>165.2</v>
+        <v>25.4</v>
       </c>
       <c r="F12" t="n">
-        <v>62.21</v>
+        <v>56.57</v>
       </c>
       <c r="G12" t="n">
-        <v>98.2</v>
+        <v>100</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -853,24 +855,26 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MAHASTEEL</t>
+          <t>STARHEALTH</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>14.48</v>
+        <v>16.19</v>
       </c>
       <c r="C13" t="n">
-        <v>211.98</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
+        <v>-3.43</v>
+      </c>
+      <c r="D13" t="n">
+        <v>7.51</v>
+      </c>
       <c r="E13" t="n">
-        <v>12.2</v>
+        <v>1407.8</v>
       </c>
       <c r="F13" t="n">
-        <v>42.9</v>
+        <v>25.78</v>
       </c>
       <c r="G13" t="n">
-        <v>71</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -887,21 +891,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TFCILTD</t>
+          <t>KOLTEPATIL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>13.55</v>
+        <v>16.07</v>
       </c>
       <c r="C14" t="n">
-        <v>91.06999999999999</v>
+        <v>6.36</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>98.3</v>
+        <v>1016.5</v>
       </c>
       <c r="F14" t="n">
-        <v>49.61</v>
+        <v>37.12</v>
       </c>
       <c r="G14" t="n">
         <v>100</v>
@@ -921,28 +925,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WELCORP</t>
+          <t>SOMATEX</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>13.37</v>
+        <v>15.55</v>
       </c>
       <c r="C15" t="n">
-        <v>89.81</v>
+        <v>47.49</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>14.9</v>
+        <v>1284.9</v>
       </c>
       <c r="F15" t="n">
-        <v>39.54</v>
+        <v>63.46</v>
       </c>
       <c r="G15" t="n">
         <v>100</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -955,24 +959,24 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MOREPENLAB</t>
+          <t>PVP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>13.09</v>
+        <v>15.5</v>
       </c>
       <c r="C16" t="n">
-        <v>32.89</v>
+        <v>56.74</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>34.1</v>
+        <v>165.2</v>
       </c>
       <c r="F16" t="n">
-        <v>54.77</v>
+        <v>62.21</v>
       </c>
       <c r="G16" t="n">
-        <v>100</v>
+        <v>98.2</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -989,21 +993,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>COMSYN</t>
+          <t>KERNEX</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13.08</v>
+        <v>15.47</v>
       </c>
       <c r="C17" t="n">
-        <v>95.59</v>
+        <v>77.31999999999999</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>20.6</v>
+        <v>800.4</v>
       </c>
       <c r="F17" t="n">
-        <v>48.74</v>
+        <v>60.32</v>
       </c>
       <c r="G17" t="n">
         <v>100</v>
@@ -1023,26 +1027,24 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SANOFI</t>
+          <t>MAHASTEEL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>12.46</v>
+        <v>14.56</v>
       </c>
       <c r="C18" t="n">
-        <v>-28.22</v>
-      </c>
-      <c r="D18" t="n">
-        <v>40.27</v>
-      </c>
+        <v>211.98</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>7.7</v>
+        <v>12.2</v>
       </c>
       <c r="F18" t="n">
-        <v>21.46</v>
+        <v>42.9</v>
       </c>
       <c r="G18" t="n">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1059,21 +1061,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RPEL</t>
+          <t>TFCILTD</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>12.44</v>
+        <v>14.14</v>
       </c>
       <c r="C19" t="n">
-        <v>88.23</v>
+        <v>91.06999999999999</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>48.7</v>
+        <v>98.3</v>
       </c>
       <c r="F19" t="n">
-        <v>51.63</v>
+        <v>49.61</v>
       </c>
       <c r="G19" t="n">
         <v>100</v>
@@ -1093,28 +1095,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>WELCORP</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>11.7</v>
+        <v>13.58</v>
       </c>
       <c r="C20" t="n">
-        <v>104.23</v>
+        <v>89.81</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>29.1</v>
+        <v>14.9</v>
       </c>
       <c r="F20" t="n">
-        <v>33.15</v>
+        <v>39.54</v>
       </c>
       <c r="G20" t="n">
         <v>100</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -1127,21 +1129,23 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SANOFI</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>11.66</v>
+        <v>13.05</v>
       </c>
       <c r="C21" t="n">
-        <v>42.79</v>
-      </c>
-      <c r="D21" t="inlineStr"/>
+        <v>-28.22</v>
+      </c>
+      <c r="D21" t="n">
+        <v>40.27</v>
+      </c>
       <c r="E21" t="n">
-        <v>34.8</v>
+        <v>7.7</v>
       </c>
       <c r="F21" t="n">
-        <v>60.4</v>
+        <v>21.46</v>
       </c>
       <c r="G21" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add real market-hours check to Live_Execution_Monitor.py - stops cleanly at close instead of continuing to refresh with stale post-market data
</commit_message>
<xml_diff>
--- a/COMPOUNDER_WATCHLIST.xlsx
+++ b/COMPOUNDER_WATCHLIST.xlsx
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>37.22</v>
+        <v>37.33</v>
       </c>
       <c r="C2" t="n">
         <v>-21.55</v>
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35.45</v>
+        <v>35.68</v>
       </c>
       <c r="C3" t="n">
         <v>-6.34</v>
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30.34</v>
+        <v>30.41</v>
       </c>
       <c r="C4" t="n">
         <v>279.21</v>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22.84</v>
+        <v>22.93</v>
       </c>
       <c r="C5" t="n">
         <v>-25.51</v>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21.49</v>
+        <v>21.61</v>
       </c>
       <c r="C6" t="n">
         <v>-12.35</v>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>21.2</v>
+        <v>21.29</v>
       </c>
       <c r="C7" t="n">
         <v>7.68</v>
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20.73</v>
+        <v>20.79</v>
       </c>
       <c r="C8" t="n">
         <v>265.44</v>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>18.97</v>
+        <v>19.03</v>
       </c>
       <c r="C9" t="n">
         <v>217.16</v>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17.17</v>
+        <v>17.18</v>
       </c>
       <c r="C10" t="n">
         <v>65.77</v>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16.76</v>
+        <v>16.84</v>
       </c>
       <c r="C11" t="n">
         <v>-23.66</v>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.19</v>
+        <v>16.21</v>
       </c>
       <c r="C13" t="n">
         <v>-3.43</v>
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.07</v>
+        <v>16.13</v>
       </c>
       <c r="C14" t="n">
         <v>6.36</v>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.55</v>
+        <v>15.64</v>
       </c>
       <c r="C15" t="n">
         <v>47.49</v>
@@ -959,24 +959,24 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PVP</t>
+          <t>KERNEX</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>15.5</v>
+        <v>15.54</v>
       </c>
       <c r="C16" t="n">
-        <v>56.74</v>
+        <v>77.31999999999999</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>165.2</v>
+        <v>800.4</v>
       </c>
       <c r="F16" t="n">
-        <v>62.21</v>
+        <v>60.32</v>
       </c>
       <c r="G16" t="n">
-        <v>98.2</v>
+        <v>100</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -993,24 +993,24 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KERNEX</t>
+          <t>PVP</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15.47</v>
+        <v>15.51</v>
       </c>
       <c r="C17" t="n">
-        <v>77.31999999999999</v>
+        <v>56.74</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>800.4</v>
+        <v>165.2</v>
       </c>
       <c r="F17" t="n">
-        <v>60.32</v>
+        <v>62.21</v>
       </c>
       <c r="G17" t="n">
-        <v>100</v>
+        <v>98.2</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>14.56</v>
+        <v>14.61</v>
       </c>
       <c r="C18" t="n">
         <v>211.98</v>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>14.14</v>
+        <v>14.17</v>
       </c>
       <c r="C19" t="n">
         <v>91.06999999999999</v>
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>13.58</v>
+        <v>13.6</v>
       </c>
       <c r="C20" t="n">
         <v>89.81</v>
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>13.05</v>
+        <v>13.1</v>
       </c>
       <c r="C21" t="n">
         <v>-28.22</v>

</xml_diff>